<commit_message>
chore(frontend): retirar comentarios internos de la plantilla
</commit_message>
<xml_diff>
--- a/frontend/public/Plantilla_presentaciones_operadoras.xlsx
+++ b/frontend/public/Plantilla_presentaciones_operadoras.xlsx
@@ -2,41 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Presentaciones" sheetId="1" r:id="R151b483b27c14f51"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="2" r:id="Rcbc94c8a787e4f18"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Presentaciones" sheetId="1" r:id="Re794285249b74979"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="2" r:id="R67d3b646878b4c2f"/>
   </x:sheets>
 </x:workbook>
-</file>
-
-<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:comments xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:authors>
-    <x:author>tc={B2ECD386-2369-4184-909C-6FBE80FBC593}</x:author>
-    <x:author>tc={52E0C7EA-6951-4AE1-B697-39C35E638B66}</x:author>
-  </x:authors>
-  <x:commentList>
-    <x:comment ref="D5" authorId="0">
-      <x:text>
-        <x:r>
-          <x:t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-    Identificador técnico opcional. Si la app exporta esta planilla, conviene conservarlo para evitar coincidencias ambiguas.</x:t>
-        </x:r>
-      </x:text>
-    </x:comment>
-    <x:comment ref="F5" authorId="1">
-      <x:text>
-        <x:r>
-          <x:t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-    Identificador técnico opcional del tipo documental. No lo modifique si viene precargado por la app.</x:t>
-        </x:r>
-      </x:text>
-    </x:comment>
-  </x:commentList>
-</x:comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
@@ -372,12 +341,6 @@
     </x:dxf>
   </x:dxfs>
 </x:styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<xltc:personList xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:person displayName="FieldService" id="{156EF50E-91D1-49BE-AC1A-A26C1DD3DA22}"/>
-</xltc:personList>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -593,17 +556,6 @@
 </a:theme>
 </file>
 
-<file path=xl/threadedcomments/threadedcomment.xml><?xml version="1.0" encoding="utf-8"?>
-<xltc:ThreadedComments xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:threadedComment ref="D5" dT="2026-09-27T23:11:29.041" personId="{156EF50E-91D1-49BE-AC1A-A26C1DD3DA22}" id="{B2ECD386-2369-4184-909C-6FBE80FBC593}">
-    <xltc:text>Identificador técnico opcional. Si la app exporta esta planilla, conviene conservarlo para evitar coincidencias ambiguas.</xltc:text>
-  </xltc:threadedComment>
-  <xltc:threadedComment ref="F5" dT="2026-09-27T23:11:29.041" personId="{156EF50E-91D1-49BE-AC1A-A26C1DD3DA22}" id="{52E0C7EA-6951-4AE1-B697-39C35E638B66}">
-    <xltc:text>Identificador técnico opcional del tipo documental. No lo modifique si viene precargado por la app.</xltc:text>
-  </xltc:threadedComment>
-</xltc:ThreadedComments>
-</file>
-
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetPr>
@@ -1554,9 +1506,8 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc2ca76cd8be24d9b"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc74b6b8acea348da"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8e137ad4398e45da"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Corregir plantilla operadoras, tests CI y UX post-auditoría Fase 4.
Observación sin fórmulas, Control en Excel ignorado al importar; sugerencias por similitud; OpenAPI y README al día.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/frontend/public/Plantilla_presentaciones_operadoras.xlsx
+++ b/frontend/public/Plantilla_presentaciones_operadoras.xlsx
@@ -635,7 +635,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N50"/>
+  <dimension ref="A1:O50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -746,6 +746,11 @@
           <t>Observación</t>
         </is>
       </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>Control</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="22" customHeight="1">
       <c r="A6" s="18" t="n"/>
@@ -761,8 +766,9 @@
       <c r="K6" s="51" t="n"/>
       <c r="L6" s="51" t="n"/>
       <c r="M6" s="17" t="n"/>
-      <c r="N6" s="20">
-        <f>IF(COUNTA(A6:M6)=0,"",IF(OR(A6="",B6="",C6="",E6="",I6=""),"Faltan campos obligatorios",IF(AND(I6="exportado",J6=""),"Falta fecha de exportación",IF(AND(OR(I6="enviado",I6="aceptado",I6="rechazado"),K6=""),"Falta fecha de presentación",IF(AND(OR(I6="aceptado",I6="rechazado"),L6=""),"Falta fecha de respuesta",IF(AND(H6&lt;&gt;"",G6&lt;&gt;"",H6&lt;G6),"Vencimiento anterior a emisión","Lista para importar"))))))</f>
+      <c r="N6" s="20" t="n"/>
+      <c r="O6">
+        <f>IF(COUNTA(A6:M6)=0,"",IF(OR(A6="",B6="",C6="",E6="",J6=""),"Faltan campos obligatorios",IF(AND(J6="exportado",K6=""),"Falta fecha de exportación",IF(AND(OR(J6="enviado",J6="aceptado",J6="rechazado"),L6=""),"Falta fecha de presentación",IF(AND(OR(J6="aceptado",J6="rechazado"),M6=""),"Falta fecha de respuesta",IF(AND(I6&lt;&gt;"",H6&lt;&gt;"",I6&lt;H6),"Vencimiento anterior a emisión","Lista para importar")))))</f>
         <v/>
       </c>
     </row>
@@ -780,8 +786,9 @@
       <c r="K7" s="51" t="n"/>
       <c r="L7" s="51" t="n"/>
       <c r="M7" s="17" t="n"/>
-      <c r="N7" s="20">
-        <f>IF(COUNTA(A7:M7)=0,"",IF(OR(A7="",B7="",C7="",E7="",I7=""),"Faltan campos obligatorios",IF(AND(I7="exportado",J7=""),"Falta fecha de exportación",IF(AND(OR(I7="enviado",I7="aceptado",I7="rechazado"),K7=""),"Falta fecha de presentación",IF(AND(OR(I7="aceptado",I7="rechazado"),L7=""),"Falta fecha de respuesta",IF(AND(H7&lt;&gt;"",G7&lt;&gt;"",H7&lt;G7),"Vencimiento anterior a emisión","Lista para importar"))))))</f>
+      <c r="N7" s="20" t="n"/>
+      <c r="O7">
+        <f>IF(COUNTA(A7:M7)=0,"",IF(OR(A7="",B7="",C7="",E7="",J7=""),"Faltan campos obligatorios",IF(AND(J7="exportado",K7=""),"Falta fecha de exportación",IF(AND(OR(J7="enviado",J7="aceptado",J7="rechazado"),L7=""),"Falta fecha de presentación",IF(AND(OR(J7="aceptado",J7="rechazado"),M7=""),"Falta fecha de respuesta",IF(AND(I7&lt;&gt;"",H7&lt;&gt;"",I7&lt;H7),"Vencimiento anterior a emisión","Lista para importar")))))</f>
         <v/>
       </c>
     </row>
@@ -799,8 +806,9 @@
       <c r="K8" s="51" t="n"/>
       <c r="L8" s="51" t="n"/>
       <c r="M8" s="17" t="n"/>
-      <c r="N8" s="20">
-        <f>IF(COUNTA(A8:M8)=0,"",IF(OR(A8="",B8="",C8="",E8="",I8=""),"Faltan campos obligatorios",IF(AND(I8="exportado",J8=""),"Falta fecha de exportación",IF(AND(OR(I8="enviado",I8="aceptado",I8="rechazado"),K8=""),"Falta fecha de presentación",IF(AND(OR(I8="aceptado",I8="rechazado"),L8=""),"Falta fecha de respuesta",IF(AND(H8&lt;&gt;"",G8&lt;&gt;"",H8&lt;G8),"Vencimiento anterior a emisión","Lista para importar"))))))</f>
+      <c r="N8" s="20" t="n"/>
+      <c r="O8">
+        <f>IF(COUNTA(A8:M8)=0,"",IF(OR(A8="",B8="",C8="",E8="",J8=""),"Faltan campos obligatorios",IF(AND(J8="exportado",K8=""),"Falta fecha de exportación",IF(AND(OR(J8="enviado",J8="aceptado",J8="rechazado"),L8=""),"Falta fecha de presentación",IF(AND(OR(J8="aceptado",J8="rechazado"),M8=""),"Falta fecha de respuesta",IF(AND(I8&lt;&gt;"",H8&lt;&gt;"",I8&lt;H8),"Vencimiento anterior a emisión","Lista para importar")))))</f>
         <v/>
       </c>
     </row>
@@ -818,8 +826,9 @@
       <c r="K9" s="51" t="n"/>
       <c r="L9" s="51" t="n"/>
       <c r="M9" s="17" t="n"/>
-      <c r="N9" s="20">
-        <f>IF(COUNTA(A9:M9)=0,"",IF(OR(A9="",B9="",C9="",E9="",I9=""),"Faltan campos obligatorios",IF(AND(I9="exportado",J9=""),"Falta fecha de exportación",IF(AND(OR(I9="enviado",I9="aceptado",I9="rechazado"),K9=""),"Falta fecha de presentación",IF(AND(OR(I9="aceptado",I9="rechazado"),L9=""),"Falta fecha de respuesta",IF(AND(H9&lt;&gt;"",G9&lt;&gt;"",H9&lt;G9),"Vencimiento anterior a emisión","Lista para importar"))))))</f>
+      <c r="N9" s="20" t="n"/>
+      <c r="O9">
+        <f>IF(COUNTA(A9:M9)=0,"",IF(OR(A9="",B9="",C9="",E9="",J9=""),"Faltan campos obligatorios",IF(AND(J9="exportado",K9=""),"Falta fecha de exportación",IF(AND(OR(J9="enviado",J9="aceptado",J9="rechazado"),L9=""),"Falta fecha de presentación",IF(AND(OR(J9="aceptado",J9="rechazado"),M9=""),"Falta fecha de respuesta",IF(AND(I9&lt;&gt;"",H9&lt;&gt;"",I9&lt;H9),"Vencimiento anterior a emisión","Lista para importar")))))</f>
         <v/>
       </c>
     </row>
@@ -837,8 +846,9 @@
       <c r="K10" s="51" t="n"/>
       <c r="L10" s="51" t="n"/>
       <c r="M10" s="17" t="n"/>
-      <c r="N10" s="20">
-        <f>IF(COUNTA(A10:M10)=0,"",IF(OR(A10="",B10="",C10="",E10="",I10=""),"Faltan campos obligatorios",IF(AND(I10="exportado",J10=""),"Falta fecha de exportación",IF(AND(OR(I10="enviado",I10="aceptado",I10="rechazado"),K10=""),"Falta fecha de presentación",IF(AND(OR(I10="aceptado",I10="rechazado"),L10=""),"Falta fecha de respuesta",IF(AND(H10&lt;&gt;"",G10&lt;&gt;"",H10&lt;G10),"Vencimiento anterior a emisión","Lista para importar"))))))</f>
+      <c r="N10" s="20" t="n"/>
+      <c r="O10">
+        <f>IF(COUNTA(A10:M10)=0,"",IF(OR(A10="",B10="",C10="",E10="",J10=""),"Faltan campos obligatorios",IF(AND(J10="exportado",K10=""),"Falta fecha de exportación",IF(AND(OR(J10="enviado",J10="aceptado",J10="rechazado"),L10=""),"Falta fecha de presentación",IF(AND(OR(J10="aceptado",J10="rechazado"),M10=""),"Falta fecha de respuesta",IF(AND(I10&lt;&gt;"",H10&lt;&gt;"",I10&lt;H10),"Vencimiento anterior a emisión","Lista para importar")))))</f>
         <v/>
       </c>
     </row>
@@ -856,8 +866,9 @@
       <c r="K11" s="51" t="n"/>
       <c r="L11" s="51" t="n"/>
       <c r="M11" s="17" t="n"/>
-      <c r="N11" s="20">
-        <f>IF(COUNTA(A11:M11)=0,"",IF(OR(A11="",B11="",C11="",E11="",I11=""),"Faltan campos obligatorios",IF(AND(I11="exportado",J11=""),"Falta fecha de exportación",IF(AND(OR(I11="enviado",I11="aceptado",I11="rechazado"),K11=""),"Falta fecha de presentación",IF(AND(OR(I11="aceptado",I11="rechazado"),L11=""),"Falta fecha de respuesta",IF(AND(H11&lt;&gt;"",G11&lt;&gt;"",H11&lt;G11),"Vencimiento anterior a emisión","Lista para importar"))))))</f>
+      <c r="N11" s="20" t="n"/>
+      <c r="O11">
+        <f>IF(COUNTA(A11:M11)=0,"",IF(OR(A11="",B11="",C11="",E11="",J11=""),"Faltan campos obligatorios",IF(AND(J11="exportado",K11=""),"Falta fecha de exportación",IF(AND(OR(J11="enviado",J11="aceptado",J11="rechazado"),L11=""),"Falta fecha de presentación",IF(AND(OR(J11="aceptado",J11="rechazado"),M11=""),"Falta fecha de respuesta",IF(AND(I11&lt;&gt;"",H11&lt;&gt;"",I11&lt;H11),"Vencimiento anterior a emisión","Lista para importar")))))</f>
         <v/>
       </c>
     </row>
@@ -875,8 +886,9 @@
       <c r="K12" s="51" t="n"/>
       <c r="L12" s="51" t="n"/>
       <c r="M12" s="17" t="n"/>
-      <c r="N12" s="20">
-        <f>IF(COUNTA(A12:M12)=0,"",IF(OR(A12="",B12="",C12="",E12="",I12=""),"Faltan campos obligatorios",IF(AND(I12="exportado",J12=""),"Falta fecha de exportación",IF(AND(OR(I12="enviado",I12="aceptado",I12="rechazado"),K12=""),"Falta fecha de presentación",IF(AND(OR(I12="aceptado",I12="rechazado"),L12=""),"Falta fecha de respuesta",IF(AND(H12&lt;&gt;"",G12&lt;&gt;"",H12&lt;G12),"Vencimiento anterior a emisión","Lista para importar"))))))</f>
+      <c r="N12" s="20" t="n"/>
+      <c r="O12">
+        <f>IF(COUNTA(A12:M12)=0,"",IF(OR(A12="",B12="",C12="",E12="",J12=""),"Faltan campos obligatorios",IF(AND(J12="exportado",K12=""),"Falta fecha de exportación",IF(AND(OR(J12="enviado",J12="aceptado",J12="rechazado"),L12=""),"Falta fecha de presentación",IF(AND(OR(J12="aceptado",J12="rechazado"),M12=""),"Falta fecha de respuesta",IF(AND(I12&lt;&gt;"",H12&lt;&gt;"",I12&lt;H12),"Vencimiento anterior a emisión","Lista para importar")))))</f>
         <v/>
       </c>
     </row>
@@ -894,8 +906,9 @@
       <c r="K13" s="51" t="n"/>
       <c r="L13" s="51" t="n"/>
       <c r="M13" s="17" t="n"/>
-      <c r="N13" s="20">
-        <f>IF(COUNTA(A13:M13)=0,"",IF(OR(A13="",B13="",C13="",E13="",I13=""),"Faltan campos obligatorios",IF(AND(I13="exportado",J13=""),"Falta fecha de exportación",IF(AND(OR(I13="enviado",I13="aceptado",I13="rechazado"),K13=""),"Falta fecha de presentación",IF(AND(OR(I13="aceptado",I13="rechazado"),L13=""),"Falta fecha de respuesta",IF(AND(H13&lt;&gt;"",G13&lt;&gt;"",H13&lt;G13),"Vencimiento anterior a emisión","Lista para importar"))))))</f>
+      <c r="N13" s="20" t="n"/>
+      <c r="O13">
+        <f>IF(COUNTA(A13:M13)=0,"",IF(OR(A13="",B13="",C13="",E13="",J13=""),"Faltan campos obligatorios",IF(AND(J13="exportado",K13=""),"Falta fecha de exportación",IF(AND(OR(J13="enviado",J13="aceptado",J13="rechazado"),L13=""),"Falta fecha de presentación",IF(AND(OR(J13="aceptado",J13="rechazado"),M13=""),"Falta fecha de respuesta",IF(AND(I13&lt;&gt;"",H13&lt;&gt;"",I13&lt;H13),"Vencimiento anterior a emisión","Lista para importar")))))</f>
         <v/>
       </c>
     </row>
@@ -913,8 +926,9 @@
       <c r="K14" s="51" t="n"/>
       <c r="L14" s="51" t="n"/>
       <c r="M14" s="17" t="n"/>
-      <c r="N14" s="20">
-        <f>IF(COUNTA(A14:M14)=0,"",IF(OR(A14="",B14="",C14="",E14="",I14=""),"Faltan campos obligatorios",IF(AND(I14="exportado",J14=""),"Falta fecha de exportación",IF(AND(OR(I14="enviado",I14="aceptado",I14="rechazado"),K14=""),"Falta fecha de presentación",IF(AND(OR(I14="aceptado",I14="rechazado"),L14=""),"Falta fecha de respuesta",IF(AND(H14&lt;&gt;"",G14&lt;&gt;"",H14&lt;G14),"Vencimiento anterior a emisión","Lista para importar"))))))</f>
+      <c r="N14" s="20" t="n"/>
+      <c r="O14">
+        <f>IF(COUNTA(A14:M14)=0,"",IF(OR(A14="",B14="",C14="",E14="",J14=""),"Faltan campos obligatorios",IF(AND(J14="exportado",K14=""),"Falta fecha de exportación",IF(AND(OR(J14="enviado",J14="aceptado",J14="rechazado"),L14=""),"Falta fecha de presentación",IF(AND(OR(J14="aceptado",J14="rechazado"),M14=""),"Falta fecha de respuesta",IF(AND(I14&lt;&gt;"",H14&lt;&gt;"",I14&lt;H14),"Vencimiento anterior a emisión","Lista para importar")))))</f>
         <v/>
       </c>
     </row>
@@ -932,8 +946,9 @@
       <c r="K15" s="51" t="n"/>
       <c r="L15" s="51" t="n"/>
       <c r="M15" s="17" t="n"/>
-      <c r="N15" s="20">
-        <f>IF(COUNTA(A15:M15)=0,"",IF(OR(A15="",B15="",C15="",E15="",I15=""),"Faltan campos obligatorios",IF(AND(I15="exportado",J15=""),"Falta fecha de exportación",IF(AND(OR(I15="enviado",I15="aceptado",I15="rechazado"),K15=""),"Falta fecha de presentación",IF(AND(OR(I15="aceptado",I15="rechazado"),L15=""),"Falta fecha de respuesta",IF(AND(H15&lt;&gt;"",G15&lt;&gt;"",H15&lt;G15),"Vencimiento anterior a emisión","Lista para importar"))))))</f>
+      <c r="N15" s="20" t="n"/>
+      <c r="O15">
+        <f>IF(COUNTA(A15:M15)=0,"",IF(OR(A15="",B15="",C15="",E15="",J15=""),"Faltan campos obligatorios",IF(AND(J15="exportado",K15=""),"Falta fecha de exportación",IF(AND(OR(J15="enviado",J15="aceptado",J15="rechazado"),L15=""),"Falta fecha de presentación",IF(AND(OR(J15="aceptado",J15="rechazado"),M15=""),"Falta fecha de respuesta",IF(AND(I15&lt;&gt;"",H15&lt;&gt;"",I15&lt;H15),"Vencimiento anterior a emisión","Lista para importar")))))</f>
         <v/>
       </c>
     </row>
@@ -951,8 +966,9 @@
       <c r="K16" s="51" t="n"/>
       <c r="L16" s="51" t="n"/>
       <c r="M16" s="17" t="n"/>
-      <c r="N16" s="20">
-        <f>IF(COUNTA(A16:M16)=0,"",IF(OR(A16="",B16="",C16="",E16="",I16=""),"Faltan campos obligatorios",IF(AND(I16="exportado",J16=""),"Falta fecha de exportación",IF(AND(OR(I16="enviado",I16="aceptado",I16="rechazado"),K16=""),"Falta fecha de presentación",IF(AND(OR(I16="aceptado",I16="rechazado"),L16=""),"Falta fecha de respuesta",IF(AND(H16&lt;&gt;"",G16&lt;&gt;"",H16&lt;G16),"Vencimiento anterior a emisión","Lista para importar"))))))</f>
+      <c r="N16" s="20" t="n"/>
+      <c r="O16">
+        <f>IF(COUNTA(A16:M16)=0,"",IF(OR(A16="",B16="",C16="",E16="",J16=""),"Faltan campos obligatorios",IF(AND(J16="exportado",K16=""),"Falta fecha de exportación",IF(AND(OR(J16="enviado",J16="aceptado",J16="rechazado"),L16=""),"Falta fecha de presentación",IF(AND(OR(J16="aceptado",J16="rechazado"),M16=""),"Falta fecha de respuesta",IF(AND(I16&lt;&gt;"",H16&lt;&gt;"",I16&lt;H16),"Vencimiento anterior a emisión","Lista para importar")))))</f>
         <v/>
       </c>
     </row>
@@ -970,8 +986,9 @@
       <c r="K17" s="51" t="n"/>
       <c r="L17" s="51" t="n"/>
       <c r="M17" s="17" t="n"/>
-      <c r="N17" s="20">
-        <f>IF(COUNTA(A17:M17)=0,"",IF(OR(A17="",B17="",C17="",E17="",I17=""),"Faltan campos obligatorios",IF(AND(I17="exportado",J17=""),"Falta fecha de exportación",IF(AND(OR(I17="enviado",I17="aceptado",I17="rechazado"),K17=""),"Falta fecha de presentación",IF(AND(OR(I17="aceptado",I17="rechazado"),L17=""),"Falta fecha de respuesta",IF(AND(H17&lt;&gt;"",G17&lt;&gt;"",H17&lt;G17),"Vencimiento anterior a emisión","Lista para importar"))))))</f>
+      <c r="N17" s="20" t="n"/>
+      <c r="O17">
+        <f>IF(COUNTA(A17:M17)=0,"",IF(OR(A17="",B17="",C17="",E17="",J17=""),"Faltan campos obligatorios",IF(AND(J17="exportado",K17=""),"Falta fecha de exportación",IF(AND(OR(J17="enviado",J17="aceptado",J17="rechazado"),L17=""),"Falta fecha de presentación",IF(AND(OR(J17="aceptado",J17="rechazado"),M17=""),"Falta fecha de respuesta",IF(AND(I17&lt;&gt;"",H17&lt;&gt;"",I17&lt;H17),"Vencimiento anterior a emisión","Lista para importar")))))</f>
         <v/>
       </c>
     </row>
@@ -989,8 +1006,9 @@
       <c r="K18" s="51" t="n"/>
       <c r="L18" s="51" t="n"/>
       <c r="M18" s="17" t="n"/>
-      <c r="N18" s="20">
-        <f>IF(COUNTA(A18:M18)=0,"",IF(OR(A18="",B18="",C18="",E18="",I18=""),"Faltan campos obligatorios",IF(AND(I18="exportado",J18=""),"Falta fecha de exportación",IF(AND(OR(I18="enviado",I18="aceptado",I18="rechazado"),K18=""),"Falta fecha de presentación",IF(AND(OR(I18="aceptado",I18="rechazado"),L18=""),"Falta fecha de respuesta",IF(AND(H18&lt;&gt;"",G18&lt;&gt;"",H18&lt;G18),"Vencimiento anterior a emisión","Lista para importar"))))))</f>
+      <c r="N18" s="20" t="n"/>
+      <c r="O18">
+        <f>IF(COUNTA(A18:M18)=0,"",IF(OR(A18="",B18="",C18="",E18="",J18=""),"Faltan campos obligatorios",IF(AND(J18="exportado",K18=""),"Falta fecha de exportación",IF(AND(OR(J18="enviado",J18="aceptado",J18="rechazado"),L18=""),"Falta fecha de presentación",IF(AND(OR(J18="aceptado",J18="rechazado"),M18=""),"Falta fecha de respuesta",IF(AND(I18&lt;&gt;"",H18&lt;&gt;"",I18&lt;H18),"Vencimiento anterior a emisión","Lista para importar")))))</f>
         <v/>
       </c>
     </row>
@@ -1008,8 +1026,9 @@
       <c r="K19" s="51" t="n"/>
       <c r="L19" s="51" t="n"/>
       <c r="M19" s="17" t="n"/>
-      <c r="N19" s="20">
-        <f>IF(COUNTA(A19:M19)=0,"",IF(OR(A19="",B19="",C19="",E19="",I19=""),"Faltan campos obligatorios",IF(AND(I19="exportado",J19=""),"Falta fecha de exportación",IF(AND(OR(I19="enviado",I19="aceptado",I19="rechazado"),K19=""),"Falta fecha de presentación",IF(AND(OR(I19="aceptado",I19="rechazado"),L19=""),"Falta fecha de respuesta",IF(AND(H19&lt;&gt;"",G19&lt;&gt;"",H19&lt;G19),"Vencimiento anterior a emisión","Lista para importar"))))))</f>
+      <c r="N19" s="20" t="n"/>
+      <c r="O19">
+        <f>IF(COUNTA(A19:M19)=0,"",IF(OR(A19="",B19="",C19="",E19="",J19=""),"Faltan campos obligatorios",IF(AND(J19="exportado",K19=""),"Falta fecha de exportación",IF(AND(OR(J19="enviado",J19="aceptado",J19="rechazado"),L19=""),"Falta fecha de presentación",IF(AND(OR(J19="aceptado",J19="rechazado"),M19=""),"Falta fecha de respuesta",IF(AND(I19&lt;&gt;"",H19&lt;&gt;"",I19&lt;H19),"Vencimiento anterior a emisión","Lista para importar")))))</f>
         <v/>
       </c>
     </row>
@@ -1027,8 +1046,9 @@
       <c r="K20" s="51" t="n"/>
       <c r="L20" s="51" t="n"/>
       <c r="M20" s="17" t="n"/>
-      <c r="N20" s="20">
-        <f>IF(COUNTA(A20:M20)=0,"",IF(OR(A20="",B20="",C20="",E20="",I20=""),"Faltan campos obligatorios",IF(AND(I20="exportado",J20=""),"Falta fecha de exportación",IF(AND(OR(I20="enviado",I20="aceptado",I20="rechazado"),K20=""),"Falta fecha de presentación",IF(AND(OR(I20="aceptado",I20="rechazado"),L20=""),"Falta fecha de respuesta",IF(AND(H20&lt;&gt;"",G20&lt;&gt;"",H20&lt;G20),"Vencimiento anterior a emisión","Lista para importar"))))))</f>
+      <c r="N20" s="20" t="n"/>
+      <c r="O20">
+        <f>IF(COUNTA(A20:M20)=0,"",IF(OR(A20="",B20="",C20="",E20="",J20=""),"Faltan campos obligatorios",IF(AND(J20="exportado",K20=""),"Falta fecha de exportación",IF(AND(OR(J20="enviado",J20="aceptado",J20="rechazado"),L20=""),"Falta fecha de presentación",IF(AND(OR(J20="aceptado",J20="rechazado"),M20=""),"Falta fecha de respuesta",IF(AND(I20&lt;&gt;"",H20&lt;&gt;"",I20&lt;H20),"Vencimiento anterior a emisión","Lista para importar")))))</f>
         <v/>
       </c>
     </row>
@@ -1046,8 +1066,9 @@
       <c r="K21" s="51" t="n"/>
       <c r="L21" s="51" t="n"/>
       <c r="M21" s="17" t="n"/>
-      <c r="N21" s="20">
-        <f>IF(COUNTA(A21:M21)=0,"",IF(OR(A21="",B21="",C21="",E21="",I21=""),"Faltan campos obligatorios",IF(AND(I21="exportado",J21=""),"Falta fecha de exportación",IF(AND(OR(I21="enviado",I21="aceptado",I21="rechazado"),K21=""),"Falta fecha de presentación",IF(AND(OR(I21="aceptado",I21="rechazado"),L21=""),"Falta fecha de respuesta",IF(AND(H21&lt;&gt;"",G21&lt;&gt;"",H21&lt;G21),"Vencimiento anterior a emisión","Lista para importar"))))))</f>
+      <c r="N21" s="20" t="n"/>
+      <c r="O21">
+        <f>IF(COUNTA(A21:M21)=0,"",IF(OR(A21="",B21="",C21="",E21="",J21=""),"Faltan campos obligatorios",IF(AND(J21="exportado",K21=""),"Falta fecha de exportación",IF(AND(OR(J21="enviado",J21="aceptado",J21="rechazado"),L21=""),"Falta fecha de presentación",IF(AND(OR(J21="aceptado",J21="rechazado"),M21=""),"Falta fecha de respuesta",IF(AND(I21&lt;&gt;"",H21&lt;&gt;"",I21&lt;H21),"Vencimiento anterior a emisión","Lista para importar")))))</f>
         <v/>
       </c>
     </row>
@@ -1065,8 +1086,9 @@
       <c r="K22" s="51" t="n"/>
       <c r="L22" s="51" t="n"/>
       <c r="M22" s="17" t="n"/>
-      <c r="N22" s="20">
-        <f>IF(COUNTA(A22:M22)=0,"",IF(OR(A22="",B22="",C22="",E22="",I22=""),"Faltan campos obligatorios",IF(AND(I22="exportado",J22=""),"Falta fecha de exportación",IF(AND(OR(I22="enviado",I22="aceptado",I22="rechazado"),K22=""),"Falta fecha de presentación",IF(AND(OR(I22="aceptado",I22="rechazado"),L22=""),"Falta fecha de respuesta",IF(AND(H22&lt;&gt;"",G22&lt;&gt;"",H22&lt;G22),"Vencimiento anterior a emisión","Lista para importar"))))))</f>
+      <c r="N22" s="20" t="n"/>
+      <c r="O22">
+        <f>IF(COUNTA(A22:M22)=0,"",IF(OR(A22="",B22="",C22="",E22="",J22=""),"Faltan campos obligatorios",IF(AND(J22="exportado",K22=""),"Falta fecha de exportación",IF(AND(OR(J22="enviado",J22="aceptado",J22="rechazado"),L22=""),"Falta fecha de presentación",IF(AND(OR(J22="aceptado",J22="rechazado"),M22=""),"Falta fecha de respuesta",IF(AND(I22&lt;&gt;"",H22&lt;&gt;"",I22&lt;H22),"Vencimiento anterior a emisión","Lista para importar")))))</f>
         <v/>
       </c>
     </row>
@@ -1084,8 +1106,9 @@
       <c r="K23" s="51" t="n"/>
       <c r="L23" s="51" t="n"/>
       <c r="M23" s="17" t="n"/>
-      <c r="N23" s="20">
-        <f>IF(COUNTA(A23:M23)=0,"",IF(OR(A23="",B23="",C23="",E23="",I23=""),"Faltan campos obligatorios",IF(AND(I23="exportado",J23=""),"Falta fecha de exportación",IF(AND(OR(I23="enviado",I23="aceptado",I23="rechazado"),K23=""),"Falta fecha de presentación",IF(AND(OR(I23="aceptado",I23="rechazado"),L23=""),"Falta fecha de respuesta",IF(AND(H23&lt;&gt;"",G23&lt;&gt;"",H23&lt;G23),"Vencimiento anterior a emisión","Lista para importar"))))))</f>
+      <c r="N23" s="20" t="n"/>
+      <c r="O23">
+        <f>IF(COUNTA(A23:M23)=0,"",IF(OR(A23="",B23="",C23="",E23="",J23=""),"Faltan campos obligatorios",IF(AND(J23="exportado",K23=""),"Falta fecha de exportación",IF(AND(OR(J23="enviado",J23="aceptado",J23="rechazado"),L23=""),"Falta fecha de presentación",IF(AND(OR(J23="aceptado",J23="rechazado"),M23=""),"Falta fecha de respuesta",IF(AND(I23&lt;&gt;"",H23&lt;&gt;"",I23&lt;H23),"Vencimiento anterior a emisión","Lista para importar")))))</f>
         <v/>
       </c>
     </row>
@@ -1103,8 +1126,9 @@
       <c r="K24" s="51" t="n"/>
       <c r="L24" s="51" t="n"/>
       <c r="M24" s="17" t="n"/>
-      <c r="N24" s="20">
-        <f>IF(COUNTA(A24:M24)=0,"",IF(OR(A24="",B24="",C24="",E24="",I24=""),"Faltan campos obligatorios",IF(AND(I24="exportado",J24=""),"Falta fecha de exportación",IF(AND(OR(I24="enviado",I24="aceptado",I24="rechazado"),K24=""),"Falta fecha de presentación",IF(AND(OR(I24="aceptado",I24="rechazado"),L24=""),"Falta fecha de respuesta",IF(AND(H24&lt;&gt;"",G24&lt;&gt;"",H24&lt;G24),"Vencimiento anterior a emisión","Lista para importar"))))))</f>
+      <c r="N24" s="20" t="n"/>
+      <c r="O24">
+        <f>IF(COUNTA(A24:M24)=0,"",IF(OR(A24="",B24="",C24="",E24="",J24=""),"Faltan campos obligatorios",IF(AND(J24="exportado",K24=""),"Falta fecha de exportación",IF(AND(OR(J24="enviado",J24="aceptado",J24="rechazado"),L24=""),"Falta fecha de presentación",IF(AND(OR(J24="aceptado",J24="rechazado"),M24=""),"Falta fecha de respuesta",IF(AND(I24&lt;&gt;"",H24&lt;&gt;"",I24&lt;H24),"Vencimiento anterior a emisión","Lista para importar")))))</f>
         <v/>
       </c>
     </row>
@@ -1122,8 +1146,9 @@
       <c r="K25" s="51" t="n"/>
       <c r="L25" s="51" t="n"/>
       <c r="M25" s="17" t="n"/>
-      <c r="N25" s="20">
-        <f>IF(COUNTA(A25:M25)=0,"",IF(OR(A25="",B25="",C25="",E25="",I25=""),"Faltan campos obligatorios",IF(AND(I25="exportado",J25=""),"Falta fecha de exportación",IF(AND(OR(I25="enviado",I25="aceptado",I25="rechazado"),K25=""),"Falta fecha de presentación",IF(AND(OR(I25="aceptado",I25="rechazado"),L25=""),"Falta fecha de respuesta",IF(AND(H25&lt;&gt;"",G25&lt;&gt;"",H25&lt;G25),"Vencimiento anterior a emisión","Lista para importar"))))))</f>
+      <c r="N25" s="20" t="n"/>
+      <c r="O25">
+        <f>IF(COUNTA(A25:M25)=0,"",IF(OR(A25="",B25="",C25="",E25="",J25=""),"Faltan campos obligatorios",IF(AND(J25="exportado",K25=""),"Falta fecha de exportación",IF(AND(OR(J25="enviado",J25="aceptado",J25="rechazado"),L25=""),"Falta fecha de presentación",IF(AND(OR(J25="aceptado",J25="rechazado"),M25=""),"Falta fecha de respuesta",IF(AND(I25&lt;&gt;"",H25&lt;&gt;"",I25&lt;H25),"Vencimiento anterior a emisión","Lista para importar")))))</f>
         <v/>
       </c>
     </row>
@@ -1141,8 +1166,9 @@
       <c r="K26" s="51" t="n"/>
       <c r="L26" s="51" t="n"/>
       <c r="M26" s="17" t="n"/>
-      <c r="N26" s="20">
-        <f>IF(COUNTA(A26:M26)=0,"",IF(OR(A26="",B26="",C26="",E26="",I26=""),"Faltan campos obligatorios",IF(AND(I26="exportado",J26=""),"Falta fecha de exportación",IF(AND(OR(I26="enviado",I26="aceptado",I26="rechazado"),K26=""),"Falta fecha de presentación",IF(AND(OR(I26="aceptado",I26="rechazado"),L26=""),"Falta fecha de respuesta",IF(AND(H26&lt;&gt;"",G26&lt;&gt;"",H26&lt;G26),"Vencimiento anterior a emisión","Lista para importar"))))))</f>
+      <c r="N26" s="20" t="n"/>
+      <c r="O26">
+        <f>IF(COUNTA(A26:M26)=0,"",IF(OR(A26="",B26="",C26="",E26="",J26=""),"Faltan campos obligatorios",IF(AND(J26="exportado",K26=""),"Falta fecha de exportación",IF(AND(OR(J26="enviado",J26="aceptado",J26="rechazado"),L26=""),"Falta fecha de presentación",IF(AND(OR(J26="aceptado",J26="rechazado"),M26=""),"Falta fecha de respuesta",IF(AND(I26&lt;&gt;"",H26&lt;&gt;"",I26&lt;H26),"Vencimiento anterior a emisión","Lista para importar")))))</f>
         <v/>
       </c>
     </row>
@@ -1160,8 +1186,9 @@
       <c r="K27" s="51" t="n"/>
       <c r="L27" s="51" t="n"/>
       <c r="M27" s="17" t="n"/>
-      <c r="N27" s="20">
-        <f>IF(COUNTA(A27:M27)=0,"",IF(OR(A27="",B27="",C27="",E27="",I27=""),"Faltan campos obligatorios",IF(AND(I27="exportado",J27=""),"Falta fecha de exportación",IF(AND(OR(I27="enviado",I27="aceptado",I27="rechazado"),K27=""),"Falta fecha de presentación",IF(AND(OR(I27="aceptado",I27="rechazado"),L27=""),"Falta fecha de respuesta",IF(AND(H27&lt;&gt;"",G27&lt;&gt;"",H27&lt;G27),"Vencimiento anterior a emisión","Lista para importar"))))))</f>
+      <c r="N27" s="20" t="n"/>
+      <c r="O27">
+        <f>IF(COUNTA(A27:M27)=0,"",IF(OR(A27="",B27="",C27="",E27="",J27=""),"Faltan campos obligatorios",IF(AND(J27="exportado",K27=""),"Falta fecha de exportación",IF(AND(OR(J27="enviado",J27="aceptado",J27="rechazado"),L27=""),"Falta fecha de presentación",IF(AND(OR(J27="aceptado",J27="rechazado"),M27=""),"Falta fecha de respuesta",IF(AND(I27&lt;&gt;"",H27&lt;&gt;"",I27&lt;H27),"Vencimiento anterior a emisión","Lista para importar")))))</f>
         <v/>
       </c>
     </row>
@@ -1179,8 +1206,9 @@
       <c r="K28" s="51" t="n"/>
       <c r="L28" s="51" t="n"/>
       <c r="M28" s="17" t="n"/>
-      <c r="N28" s="20">
-        <f>IF(COUNTA(A28:M28)=0,"",IF(OR(A28="",B28="",C28="",E28="",I28=""),"Faltan campos obligatorios",IF(AND(I28="exportado",J28=""),"Falta fecha de exportación",IF(AND(OR(I28="enviado",I28="aceptado",I28="rechazado"),K28=""),"Falta fecha de presentación",IF(AND(OR(I28="aceptado",I28="rechazado"),L28=""),"Falta fecha de respuesta",IF(AND(H28&lt;&gt;"",G28&lt;&gt;"",H28&lt;G28),"Vencimiento anterior a emisión","Lista para importar"))))))</f>
+      <c r="N28" s="20" t="n"/>
+      <c r="O28">
+        <f>IF(COUNTA(A28:M28)=0,"",IF(OR(A28="",B28="",C28="",E28="",J28=""),"Faltan campos obligatorios",IF(AND(J28="exportado",K28=""),"Falta fecha de exportación",IF(AND(OR(J28="enviado",J28="aceptado",J28="rechazado"),L28=""),"Falta fecha de presentación",IF(AND(OR(J28="aceptado",J28="rechazado"),M28=""),"Falta fecha de respuesta",IF(AND(I28&lt;&gt;"",H28&lt;&gt;"",I28&lt;H28),"Vencimiento anterior a emisión","Lista para importar")))))</f>
         <v/>
       </c>
     </row>
@@ -1198,8 +1226,9 @@
       <c r="K29" s="51" t="n"/>
       <c r="L29" s="51" t="n"/>
       <c r="M29" s="17" t="n"/>
-      <c r="N29" s="20">
-        <f>IF(COUNTA(A29:M29)=0,"",IF(OR(A29="",B29="",C29="",E29="",I29=""),"Faltan campos obligatorios",IF(AND(I29="exportado",J29=""),"Falta fecha de exportación",IF(AND(OR(I29="enviado",I29="aceptado",I29="rechazado"),K29=""),"Falta fecha de presentación",IF(AND(OR(I29="aceptado",I29="rechazado"),L29=""),"Falta fecha de respuesta",IF(AND(H29&lt;&gt;"",G29&lt;&gt;"",H29&lt;G29),"Vencimiento anterior a emisión","Lista para importar"))))))</f>
+      <c r="N29" s="20" t="n"/>
+      <c r="O29">
+        <f>IF(COUNTA(A29:M29)=0,"",IF(OR(A29="",B29="",C29="",E29="",J29=""),"Faltan campos obligatorios",IF(AND(J29="exportado",K29=""),"Falta fecha de exportación",IF(AND(OR(J29="enviado",J29="aceptado",J29="rechazado"),L29=""),"Falta fecha de presentación",IF(AND(OR(J29="aceptado",J29="rechazado"),M29=""),"Falta fecha de respuesta",IF(AND(I29&lt;&gt;"",H29&lt;&gt;"",I29&lt;H29),"Vencimiento anterior a emisión","Lista para importar")))))</f>
         <v/>
       </c>
     </row>
@@ -1217,8 +1246,9 @@
       <c r="K30" s="51" t="n"/>
       <c r="L30" s="51" t="n"/>
       <c r="M30" s="17" t="n"/>
-      <c r="N30" s="20">
-        <f>IF(COUNTA(A30:M30)=0,"",IF(OR(A30="",B30="",C30="",E30="",I30=""),"Faltan campos obligatorios",IF(AND(I30="exportado",J30=""),"Falta fecha de exportación",IF(AND(OR(I30="enviado",I30="aceptado",I30="rechazado"),K30=""),"Falta fecha de presentación",IF(AND(OR(I30="aceptado",I30="rechazado"),L30=""),"Falta fecha de respuesta",IF(AND(H30&lt;&gt;"",G30&lt;&gt;"",H30&lt;G30),"Vencimiento anterior a emisión","Lista para importar"))))))</f>
+      <c r="N30" s="20" t="n"/>
+      <c r="O30">
+        <f>IF(COUNTA(A30:M30)=0,"",IF(OR(A30="",B30="",C30="",E30="",J30=""),"Faltan campos obligatorios",IF(AND(J30="exportado",K30=""),"Falta fecha de exportación",IF(AND(OR(J30="enviado",J30="aceptado",J30="rechazado"),L30=""),"Falta fecha de presentación",IF(AND(OR(J30="aceptado",J30="rechazado"),M30=""),"Falta fecha de respuesta",IF(AND(I30&lt;&gt;"",H30&lt;&gt;"",I30&lt;H30),"Vencimiento anterior a emisión","Lista para importar")))))</f>
         <v/>
       </c>
     </row>
@@ -1236,8 +1266,9 @@
       <c r="K31" s="51" t="n"/>
       <c r="L31" s="51" t="n"/>
       <c r="M31" s="17" t="n"/>
-      <c r="N31" s="20">
-        <f>IF(COUNTA(A31:M31)=0,"",IF(OR(A31="",B31="",C31="",E31="",I31=""),"Faltan campos obligatorios",IF(AND(I31="exportado",J31=""),"Falta fecha de exportación",IF(AND(OR(I31="enviado",I31="aceptado",I31="rechazado"),K31=""),"Falta fecha de presentación",IF(AND(OR(I31="aceptado",I31="rechazado"),L31=""),"Falta fecha de respuesta",IF(AND(H31&lt;&gt;"",G31&lt;&gt;"",H31&lt;G31),"Vencimiento anterior a emisión","Lista para importar"))))))</f>
+      <c r="N31" s="20" t="n"/>
+      <c r="O31">
+        <f>IF(COUNTA(A31:M31)=0,"",IF(OR(A31="",B31="",C31="",E31="",J31=""),"Faltan campos obligatorios",IF(AND(J31="exportado",K31=""),"Falta fecha de exportación",IF(AND(OR(J31="enviado",J31="aceptado",J31="rechazado"),L31=""),"Falta fecha de presentación",IF(AND(OR(J31="aceptado",J31="rechazado"),M31=""),"Falta fecha de respuesta",IF(AND(I31&lt;&gt;"",H31&lt;&gt;"",I31&lt;H31),"Vencimiento anterior a emisión","Lista para importar")))))</f>
         <v/>
       </c>
     </row>
@@ -1255,8 +1286,9 @@
       <c r="K32" s="51" t="n"/>
       <c r="L32" s="51" t="n"/>
       <c r="M32" s="17" t="n"/>
-      <c r="N32" s="20">
-        <f>IF(COUNTA(A32:M32)=0,"",IF(OR(A32="",B32="",C32="",E32="",I32=""),"Faltan campos obligatorios",IF(AND(I32="exportado",J32=""),"Falta fecha de exportación",IF(AND(OR(I32="enviado",I32="aceptado",I32="rechazado"),K32=""),"Falta fecha de presentación",IF(AND(OR(I32="aceptado",I32="rechazado"),L32=""),"Falta fecha de respuesta",IF(AND(H32&lt;&gt;"",G32&lt;&gt;"",H32&lt;G32),"Vencimiento anterior a emisión","Lista para importar"))))))</f>
+      <c r="N32" s="20" t="n"/>
+      <c r="O32">
+        <f>IF(COUNTA(A32:M32)=0,"",IF(OR(A32="",B32="",C32="",E32="",J32=""),"Faltan campos obligatorios",IF(AND(J32="exportado",K32=""),"Falta fecha de exportación",IF(AND(OR(J32="enviado",J32="aceptado",J32="rechazado"),L32=""),"Falta fecha de presentación",IF(AND(OR(J32="aceptado",J32="rechazado"),M32=""),"Falta fecha de respuesta",IF(AND(I32&lt;&gt;"",H32&lt;&gt;"",I32&lt;H32),"Vencimiento anterior a emisión","Lista para importar")))))</f>
         <v/>
       </c>
     </row>
@@ -1274,8 +1306,9 @@
       <c r="K33" s="51" t="n"/>
       <c r="L33" s="51" t="n"/>
       <c r="M33" s="17" t="n"/>
-      <c r="N33" s="20">
-        <f>IF(COUNTA(A33:M33)=0,"",IF(OR(A33="",B33="",C33="",E33="",I33=""),"Faltan campos obligatorios",IF(AND(I33="exportado",J33=""),"Falta fecha de exportación",IF(AND(OR(I33="enviado",I33="aceptado",I33="rechazado"),K33=""),"Falta fecha de presentación",IF(AND(OR(I33="aceptado",I33="rechazado"),L33=""),"Falta fecha de respuesta",IF(AND(H33&lt;&gt;"",G33&lt;&gt;"",H33&lt;G33),"Vencimiento anterior a emisión","Lista para importar"))))))</f>
+      <c r="N33" s="20" t="n"/>
+      <c r="O33">
+        <f>IF(COUNTA(A33:M33)=0,"",IF(OR(A33="",B33="",C33="",E33="",J33=""),"Faltan campos obligatorios",IF(AND(J33="exportado",K33=""),"Falta fecha de exportación",IF(AND(OR(J33="enviado",J33="aceptado",J33="rechazado"),L33=""),"Falta fecha de presentación",IF(AND(OR(J33="aceptado",J33="rechazado"),M33=""),"Falta fecha de respuesta",IF(AND(I33&lt;&gt;"",H33&lt;&gt;"",I33&lt;H33),"Vencimiento anterior a emisión","Lista para importar")))))</f>
         <v/>
       </c>
     </row>
@@ -1293,8 +1326,9 @@
       <c r="K34" s="51" t="n"/>
       <c r="L34" s="51" t="n"/>
       <c r="M34" s="17" t="n"/>
-      <c r="N34" s="20">
-        <f>IF(COUNTA(A34:M34)=0,"",IF(OR(A34="",B34="",C34="",E34="",I34=""),"Faltan campos obligatorios",IF(AND(I34="exportado",J34=""),"Falta fecha de exportación",IF(AND(OR(I34="enviado",I34="aceptado",I34="rechazado"),K34=""),"Falta fecha de presentación",IF(AND(OR(I34="aceptado",I34="rechazado"),L34=""),"Falta fecha de respuesta",IF(AND(H34&lt;&gt;"",G34&lt;&gt;"",H34&lt;G34),"Vencimiento anterior a emisión","Lista para importar"))))))</f>
+      <c r="N34" s="20" t="n"/>
+      <c r="O34">
+        <f>IF(COUNTA(A34:M34)=0,"",IF(OR(A34="",B34="",C34="",E34="",J34=""),"Faltan campos obligatorios",IF(AND(J34="exportado",K34=""),"Falta fecha de exportación",IF(AND(OR(J34="enviado",J34="aceptado",J34="rechazado"),L34=""),"Falta fecha de presentación",IF(AND(OR(J34="aceptado",J34="rechazado"),M34=""),"Falta fecha de respuesta",IF(AND(I34&lt;&gt;"",H34&lt;&gt;"",I34&lt;H34),"Vencimiento anterior a emisión","Lista para importar")))))</f>
         <v/>
       </c>
     </row>
@@ -1312,8 +1346,9 @@
       <c r="K35" s="51" t="n"/>
       <c r="L35" s="51" t="n"/>
       <c r="M35" s="17" t="n"/>
-      <c r="N35" s="20">
-        <f>IF(COUNTA(A35:M35)=0,"",IF(OR(A35="",B35="",C35="",E35="",I35=""),"Faltan campos obligatorios",IF(AND(I35="exportado",J35=""),"Falta fecha de exportación",IF(AND(OR(I35="enviado",I35="aceptado",I35="rechazado"),K35=""),"Falta fecha de presentación",IF(AND(OR(I35="aceptado",I35="rechazado"),L35=""),"Falta fecha de respuesta",IF(AND(H35&lt;&gt;"",G35&lt;&gt;"",H35&lt;G35),"Vencimiento anterior a emisión","Lista para importar"))))))</f>
+      <c r="N35" s="20" t="n"/>
+      <c r="O35">
+        <f>IF(COUNTA(A35:M35)=0,"",IF(OR(A35="",B35="",C35="",E35="",J35=""),"Faltan campos obligatorios",IF(AND(J35="exportado",K35=""),"Falta fecha de exportación",IF(AND(OR(J35="enviado",J35="aceptado",J35="rechazado"),L35=""),"Falta fecha de presentación",IF(AND(OR(J35="aceptado",J35="rechazado"),M35=""),"Falta fecha de respuesta",IF(AND(I35&lt;&gt;"",H35&lt;&gt;"",I35&lt;H35),"Vencimiento anterior a emisión","Lista para importar")))))</f>
         <v/>
       </c>
     </row>
@@ -1331,8 +1366,9 @@
       <c r="K36" s="51" t="n"/>
       <c r="L36" s="51" t="n"/>
       <c r="M36" s="17" t="n"/>
-      <c r="N36" s="20">
-        <f>IF(COUNTA(A36:M36)=0,"",IF(OR(A36="",B36="",C36="",E36="",I36=""),"Faltan campos obligatorios",IF(AND(I36="exportado",J36=""),"Falta fecha de exportación",IF(AND(OR(I36="enviado",I36="aceptado",I36="rechazado"),K36=""),"Falta fecha de presentación",IF(AND(OR(I36="aceptado",I36="rechazado"),L36=""),"Falta fecha de respuesta",IF(AND(H36&lt;&gt;"",G36&lt;&gt;"",H36&lt;G36),"Vencimiento anterior a emisión","Lista para importar"))))))</f>
+      <c r="N36" s="20" t="n"/>
+      <c r="O36">
+        <f>IF(COUNTA(A36:M36)=0,"",IF(OR(A36="",B36="",C36="",E36="",J36=""),"Faltan campos obligatorios",IF(AND(J36="exportado",K36=""),"Falta fecha de exportación",IF(AND(OR(J36="enviado",J36="aceptado",J36="rechazado"),L36=""),"Falta fecha de presentación",IF(AND(OR(J36="aceptado",J36="rechazado"),M36=""),"Falta fecha de respuesta",IF(AND(I36&lt;&gt;"",H36&lt;&gt;"",I36&lt;H36),"Vencimiento anterior a emisión","Lista para importar")))))</f>
         <v/>
       </c>
     </row>
@@ -1350,8 +1386,9 @@
       <c r="K37" s="51" t="n"/>
       <c r="L37" s="51" t="n"/>
       <c r="M37" s="17" t="n"/>
-      <c r="N37" s="20">
-        <f>IF(COUNTA(A37:M37)=0,"",IF(OR(A37="",B37="",C37="",E37="",I37=""),"Faltan campos obligatorios",IF(AND(I37="exportado",J37=""),"Falta fecha de exportación",IF(AND(OR(I37="enviado",I37="aceptado",I37="rechazado"),K37=""),"Falta fecha de presentación",IF(AND(OR(I37="aceptado",I37="rechazado"),L37=""),"Falta fecha de respuesta",IF(AND(H37&lt;&gt;"",G37&lt;&gt;"",H37&lt;G37),"Vencimiento anterior a emisión","Lista para importar"))))))</f>
+      <c r="N37" s="20" t="n"/>
+      <c r="O37">
+        <f>IF(COUNTA(A37:M37)=0,"",IF(OR(A37="",B37="",C37="",E37="",J37=""),"Faltan campos obligatorios",IF(AND(J37="exportado",K37=""),"Falta fecha de exportación",IF(AND(OR(J37="enviado",J37="aceptado",J37="rechazado"),L37=""),"Falta fecha de presentación",IF(AND(OR(J37="aceptado",J37="rechazado"),M37=""),"Falta fecha de respuesta",IF(AND(I37&lt;&gt;"",H37&lt;&gt;"",I37&lt;H37),"Vencimiento anterior a emisión","Lista para importar")))))</f>
         <v/>
       </c>
     </row>
@@ -1369,8 +1406,9 @@
       <c r="K38" s="51" t="n"/>
       <c r="L38" s="51" t="n"/>
       <c r="M38" s="17" t="n"/>
-      <c r="N38" s="20">
-        <f>IF(COUNTA(A38:M38)=0,"",IF(OR(A38="",B38="",C38="",E38="",I38=""),"Faltan campos obligatorios",IF(AND(I38="exportado",J38=""),"Falta fecha de exportación",IF(AND(OR(I38="enviado",I38="aceptado",I38="rechazado"),K38=""),"Falta fecha de presentación",IF(AND(OR(I38="aceptado",I38="rechazado"),L38=""),"Falta fecha de respuesta",IF(AND(H38&lt;&gt;"",G38&lt;&gt;"",H38&lt;G38),"Vencimiento anterior a emisión","Lista para importar"))))))</f>
+      <c r="N38" s="20" t="n"/>
+      <c r="O38">
+        <f>IF(COUNTA(A38:M38)=0,"",IF(OR(A38="",B38="",C38="",E38="",J38=""),"Faltan campos obligatorios",IF(AND(J38="exportado",K38=""),"Falta fecha de exportación",IF(AND(OR(J38="enviado",J38="aceptado",J38="rechazado"),L38=""),"Falta fecha de presentación",IF(AND(OR(J38="aceptado",J38="rechazado"),M38=""),"Falta fecha de respuesta",IF(AND(I38&lt;&gt;"",H38&lt;&gt;"",I38&lt;H38),"Vencimiento anterior a emisión","Lista para importar")))))</f>
         <v/>
       </c>
     </row>
@@ -1388,8 +1426,9 @@
       <c r="K39" s="51" t="n"/>
       <c r="L39" s="51" t="n"/>
       <c r="M39" s="17" t="n"/>
-      <c r="N39" s="20">
-        <f>IF(COUNTA(A39:M39)=0,"",IF(OR(A39="",B39="",C39="",E39="",I39=""),"Faltan campos obligatorios",IF(AND(I39="exportado",J39=""),"Falta fecha de exportación",IF(AND(OR(I39="enviado",I39="aceptado",I39="rechazado"),K39=""),"Falta fecha de presentación",IF(AND(OR(I39="aceptado",I39="rechazado"),L39=""),"Falta fecha de respuesta",IF(AND(H39&lt;&gt;"",G39&lt;&gt;"",H39&lt;G39),"Vencimiento anterior a emisión","Lista para importar"))))))</f>
+      <c r="N39" s="20" t="n"/>
+      <c r="O39">
+        <f>IF(COUNTA(A39:M39)=0,"",IF(OR(A39="",B39="",C39="",E39="",J39=""),"Faltan campos obligatorios",IF(AND(J39="exportado",K39=""),"Falta fecha de exportación",IF(AND(OR(J39="enviado",J39="aceptado",J39="rechazado"),L39=""),"Falta fecha de presentación",IF(AND(OR(J39="aceptado",J39="rechazado"),M39=""),"Falta fecha de respuesta",IF(AND(I39&lt;&gt;"",H39&lt;&gt;"",I39&lt;H39),"Vencimiento anterior a emisión","Lista para importar")))))</f>
         <v/>
       </c>
     </row>
@@ -1407,8 +1446,9 @@
       <c r="K40" s="51" t="n"/>
       <c r="L40" s="51" t="n"/>
       <c r="M40" s="17" t="n"/>
-      <c r="N40" s="20">
-        <f>IF(COUNTA(A40:M40)=0,"",IF(OR(A40="",B40="",C40="",E40="",I40=""),"Faltan campos obligatorios",IF(AND(I40="exportado",J40=""),"Falta fecha de exportación",IF(AND(OR(I40="enviado",I40="aceptado",I40="rechazado"),K40=""),"Falta fecha de presentación",IF(AND(OR(I40="aceptado",I40="rechazado"),L40=""),"Falta fecha de respuesta",IF(AND(H40&lt;&gt;"",G40&lt;&gt;"",H40&lt;G40),"Vencimiento anterior a emisión","Lista para importar"))))))</f>
+      <c r="N40" s="20" t="n"/>
+      <c r="O40">
+        <f>IF(COUNTA(A40:M40)=0,"",IF(OR(A40="",B40="",C40="",E40="",J40=""),"Faltan campos obligatorios",IF(AND(J40="exportado",K40=""),"Falta fecha de exportación",IF(AND(OR(J40="enviado",J40="aceptado",J40="rechazado"),L40=""),"Falta fecha de presentación",IF(AND(OR(J40="aceptado",J40="rechazado"),M40=""),"Falta fecha de respuesta",IF(AND(I40&lt;&gt;"",H40&lt;&gt;"",I40&lt;H40),"Vencimiento anterior a emisión","Lista para importar")))))</f>
         <v/>
       </c>
     </row>
@@ -1426,8 +1466,9 @@
       <c r="K41" s="51" t="n"/>
       <c r="L41" s="51" t="n"/>
       <c r="M41" s="17" t="n"/>
-      <c r="N41" s="20">
-        <f>IF(COUNTA(A41:M41)=0,"",IF(OR(A41="",B41="",C41="",E41="",I41=""),"Faltan campos obligatorios",IF(AND(I41="exportado",J41=""),"Falta fecha de exportación",IF(AND(OR(I41="enviado",I41="aceptado",I41="rechazado"),K41=""),"Falta fecha de presentación",IF(AND(OR(I41="aceptado",I41="rechazado"),L41=""),"Falta fecha de respuesta",IF(AND(H41&lt;&gt;"",G41&lt;&gt;"",H41&lt;G41),"Vencimiento anterior a emisión","Lista para importar"))))))</f>
+      <c r="N41" s="20" t="n"/>
+      <c r="O41">
+        <f>IF(COUNTA(A41:M41)=0,"",IF(OR(A41="",B41="",C41="",E41="",J41=""),"Faltan campos obligatorios",IF(AND(J41="exportado",K41=""),"Falta fecha de exportación",IF(AND(OR(J41="enviado",J41="aceptado",J41="rechazado"),L41=""),"Falta fecha de presentación",IF(AND(OR(J41="aceptado",J41="rechazado"),M41=""),"Falta fecha de respuesta",IF(AND(I41&lt;&gt;"",H41&lt;&gt;"",I41&lt;H41),"Vencimiento anterior a emisión","Lista para importar")))))</f>
         <v/>
       </c>
     </row>
@@ -1445,8 +1486,9 @@
       <c r="K42" s="51" t="n"/>
       <c r="L42" s="51" t="n"/>
       <c r="M42" s="17" t="n"/>
-      <c r="N42" s="20">
-        <f>IF(COUNTA(A42:M42)=0,"",IF(OR(A42="",B42="",C42="",E42="",I42=""),"Faltan campos obligatorios",IF(AND(I42="exportado",J42=""),"Falta fecha de exportación",IF(AND(OR(I42="enviado",I42="aceptado",I42="rechazado"),K42=""),"Falta fecha de presentación",IF(AND(OR(I42="aceptado",I42="rechazado"),L42=""),"Falta fecha de respuesta",IF(AND(H42&lt;&gt;"",G42&lt;&gt;"",H42&lt;G42),"Vencimiento anterior a emisión","Lista para importar"))))))</f>
+      <c r="N42" s="20" t="n"/>
+      <c r="O42">
+        <f>IF(COUNTA(A42:M42)=0,"",IF(OR(A42="",B42="",C42="",E42="",J42=""),"Faltan campos obligatorios",IF(AND(J42="exportado",K42=""),"Falta fecha de exportación",IF(AND(OR(J42="enviado",J42="aceptado",J42="rechazado"),L42=""),"Falta fecha de presentación",IF(AND(OR(J42="aceptado",J42="rechazado"),M42=""),"Falta fecha de respuesta",IF(AND(I42&lt;&gt;"",H42&lt;&gt;"",I42&lt;H42),"Vencimiento anterior a emisión","Lista para importar")))))</f>
         <v/>
       </c>
     </row>
@@ -1464,8 +1506,9 @@
       <c r="K43" s="51" t="n"/>
       <c r="L43" s="51" t="n"/>
       <c r="M43" s="17" t="n"/>
-      <c r="N43" s="20">
-        <f>IF(COUNTA(A43:M43)=0,"",IF(OR(A43="",B43="",C43="",E43="",I43=""),"Faltan campos obligatorios",IF(AND(I43="exportado",J43=""),"Falta fecha de exportación",IF(AND(OR(I43="enviado",I43="aceptado",I43="rechazado"),K43=""),"Falta fecha de presentación",IF(AND(OR(I43="aceptado",I43="rechazado"),L43=""),"Falta fecha de respuesta",IF(AND(H43&lt;&gt;"",G43&lt;&gt;"",H43&lt;G43),"Vencimiento anterior a emisión","Lista para importar"))))))</f>
+      <c r="N43" s="20" t="n"/>
+      <c r="O43">
+        <f>IF(COUNTA(A43:M43)=0,"",IF(OR(A43="",B43="",C43="",E43="",J43=""),"Faltan campos obligatorios",IF(AND(J43="exportado",K43=""),"Falta fecha de exportación",IF(AND(OR(J43="enviado",J43="aceptado",J43="rechazado"),L43=""),"Falta fecha de presentación",IF(AND(OR(J43="aceptado",J43="rechazado"),M43=""),"Falta fecha de respuesta",IF(AND(I43&lt;&gt;"",H43&lt;&gt;"",I43&lt;H43),"Vencimiento anterior a emisión","Lista para importar")))))</f>
         <v/>
       </c>
     </row>
@@ -1483,8 +1526,9 @@
       <c r="K44" s="51" t="n"/>
       <c r="L44" s="51" t="n"/>
       <c r="M44" s="17" t="n"/>
-      <c r="N44" s="20">
-        <f>IF(COUNTA(A44:M44)=0,"",IF(OR(A44="",B44="",C44="",E44="",I44=""),"Faltan campos obligatorios",IF(AND(I44="exportado",J44=""),"Falta fecha de exportación",IF(AND(OR(I44="enviado",I44="aceptado",I44="rechazado"),K44=""),"Falta fecha de presentación",IF(AND(OR(I44="aceptado",I44="rechazado"),L44=""),"Falta fecha de respuesta",IF(AND(H44&lt;&gt;"",G44&lt;&gt;"",H44&lt;G44),"Vencimiento anterior a emisión","Lista para importar"))))))</f>
+      <c r="N44" s="20" t="n"/>
+      <c r="O44">
+        <f>IF(COUNTA(A44:M44)=0,"",IF(OR(A44="",B44="",C44="",E44="",J44=""),"Faltan campos obligatorios",IF(AND(J44="exportado",K44=""),"Falta fecha de exportación",IF(AND(OR(J44="enviado",J44="aceptado",J44="rechazado"),L44=""),"Falta fecha de presentación",IF(AND(OR(J44="aceptado",J44="rechazado"),M44=""),"Falta fecha de respuesta",IF(AND(I44&lt;&gt;"",H44&lt;&gt;"",I44&lt;H44),"Vencimiento anterior a emisión","Lista para importar")))))</f>
         <v/>
       </c>
     </row>
@@ -1502,8 +1546,9 @@
       <c r="K45" s="51" t="n"/>
       <c r="L45" s="51" t="n"/>
       <c r="M45" s="17" t="n"/>
-      <c r="N45" s="20">
-        <f>IF(COUNTA(A45:M45)=0,"",IF(OR(A45="",B45="",C45="",E45="",I45=""),"Faltan campos obligatorios",IF(AND(I45="exportado",J45=""),"Falta fecha de exportación",IF(AND(OR(I45="enviado",I45="aceptado",I45="rechazado"),K45=""),"Falta fecha de presentación",IF(AND(OR(I45="aceptado",I45="rechazado"),L45=""),"Falta fecha de respuesta",IF(AND(H45&lt;&gt;"",G45&lt;&gt;"",H45&lt;G45),"Vencimiento anterior a emisión","Lista para importar"))))))</f>
+      <c r="N45" s="20" t="n"/>
+      <c r="O45">
+        <f>IF(COUNTA(A45:M45)=0,"",IF(OR(A45="",B45="",C45="",E45="",J45=""),"Faltan campos obligatorios",IF(AND(J45="exportado",K45=""),"Falta fecha de exportación",IF(AND(OR(J45="enviado",J45="aceptado",J45="rechazado"),L45=""),"Falta fecha de presentación",IF(AND(OR(J45="aceptado",J45="rechazado"),M45=""),"Falta fecha de respuesta",IF(AND(I45&lt;&gt;"",H45&lt;&gt;"",I45&lt;H45),"Vencimiento anterior a emisión","Lista para importar")))))</f>
         <v/>
       </c>
     </row>
@@ -1521,8 +1566,9 @@
       <c r="K46" s="51" t="n"/>
       <c r="L46" s="51" t="n"/>
       <c r="M46" s="17" t="n"/>
-      <c r="N46" s="20">
-        <f>IF(COUNTA(A46:M46)=0,"",IF(OR(A46="",B46="",C46="",E46="",I46=""),"Faltan campos obligatorios",IF(AND(I46="exportado",J46=""),"Falta fecha de exportación",IF(AND(OR(I46="enviado",I46="aceptado",I46="rechazado"),K46=""),"Falta fecha de presentación",IF(AND(OR(I46="aceptado",I46="rechazado"),L46=""),"Falta fecha de respuesta",IF(AND(H46&lt;&gt;"",G46&lt;&gt;"",H46&lt;G46),"Vencimiento anterior a emisión","Lista para importar"))))))</f>
+      <c r="N46" s="20" t="n"/>
+      <c r="O46">
+        <f>IF(COUNTA(A46:M46)=0,"",IF(OR(A46="",B46="",C46="",E46="",J46=""),"Faltan campos obligatorios",IF(AND(J46="exportado",K46=""),"Falta fecha de exportación",IF(AND(OR(J46="enviado",J46="aceptado",J46="rechazado"),L46=""),"Falta fecha de presentación",IF(AND(OR(J46="aceptado",J46="rechazado"),M46=""),"Falta fecha de respuesta",IF(AND(I46&lt;&gt;"",H46&lt;&gt;"",I46&lt;H46),"Vencimiento anterior a emisión","Lista para importar")))))</f>
         <v/>
       </c>
     </row>
@@ -1540,8 +1586,9 @@
       <c r="K47" s="51" t="n"/>
       <c r="L47" s="51" t="n"/>
       <c r="M47" s="17" t="n"/>
-      <c r="N47" s="20">
-        <f>IF(COUNTA(A47:M47)=0,"",IF(OR(A47="",B47="",C47="",E47="",I47=""),"Faltan campos obligatorios",IF(AND(I47="exportado",J47=""),"Falta fecha de exportación",IF(AND(OR(I47="enviado",I47="aceptado",I47="rechazado"),K47=""),"Falta fecha de presentación",IF(AND(OR(I47="aceptado",I47="rechazado"),L47=""),"Falta fecha de respuesta",IF(AND(H47&lt;&gt;"",G47&lt;&gt;"",H47&lt;G47),"Vencimiento anterior a emisión","Lista para importar"))))))</f>
+      <c r="N47" s="20" t="n"/>
+      <c r="O47">
+        <f>IF(COUNTA(A47:M47)=0,"",IF(OR(A47="",B47="",C47="",E47="",J47=""),"Faltan campos obligatorios",IF(AND(J47="exportado",K47=""),"Falta fecha de exportación",IF(AND(OR(J47="enviado",J47="aceptado",J47="rechazado"),L47=""),"Falta fecha de presentación",IF(AND(OR(J47="aceptado",J47="rechazado"),M47=""),"Falta fecha de respuesta",IF(AND(I47&lt;&gt;"",H47&lt;&gt;"",I47&lt;H47),"Vencimiento anterior a emisión","Lista para importar")))))</f>
         <v/>
       </c>
     </row>
@@ -1559,8 +1606,9 @@
       <c r="K48" s="51" t="n"/>
       <c r="L48" s="51" t="n"/>
       <c r="M48" s="17" t="n"/>
-      <c r="N48" s="20">
-        <f>IF(COUNTA(A48:M48)=0,"",IF(OR(A48="",B48="",C48="",E48="",I48=""),"Faltan campos obligatorios",IF(AND(I48="exportado",J48=""),"Falta fecha de exportación",IF(AND(OR(I48="enviado",I48="aceptado",I48="rechazado"),K48=""),"Falta fecha de presentación",IF(AND(OR(I48="aceptado",I48="rechazado"),L48=""),"Falta fecha de respuesta",IF(AND(H48&lt;&gt;"",G48&lt;&gt;"",H48&lt;G48),"Vencimiento anterior a emisión","Lista para importar"))))))</f>
+      <c r="N48" s="20" t="n"/>
+      <c r="O48">
+        <f>IF(COUNTA(A48:M48)=0,"",IF(OR(A48="",B48="",C48="",E48="",J48=""),"Faltan campos obligatorios",IF(AND(J48="exportado",K48=""),"Falta fecha de exportación",IF(AND(OR(J48="enviado",J48="aceptado",J48="rechazado"),L48=""),"Falta fecha de presentación",IF(AND(OR(J48="aceptado",J48="rechazado"),M48=""),"Falta fecha de respuesta",IF(AND(I48&lt;&gt;"",H48&lt;&gt;"",I48&lt;H48),"Vencimiento anterior a emisión","Lista para importar")))))</f>
         <v/>
       </c>
     </row>
@@ -1578,8 +1626,9 @@
       <c r="K49" s="51" t="n"/>
       <c r="L49" s="51" t="n"/>
       <c r="M49" s="17" t="n"/>
-      <c r="N49" s="20">
-        <f>IF(COUNTA(A49:M49)=0,"",IF(OR(A49="",B49="",C49="",E49="",I49=""),"Faltan campos obligatorios",IF(AND(I49="exportado",J49=""),"Falta fecha de exportación",IF(AND(OR(I49="enviado",I49="aceptado",I49="rechazado"),K49=""),"Falta fecha de presentación",IF(AND(OR(I49="aceptado",I49="rechazado"),L49=""),"Falta fecha de respuesta",IF(AND(H49&lt;&gt;"",G49&lt;&gt;"",H49&lt;G49),"Vencimiento anterior a emisión","Lista para importar"))))))</f>
+      <c r="N49" s="20" t="n"/>
+      <c r="O49">
+        <f>IF(COUNTA(A49:M49)=0,"",IF(OR(A49="",B49="",C49="",E49="",J49=""),"Faltan campos obligatorios",IF(AND(J49="exportado",K49=""),"Falta fecha de exportación",IF(AND(OR(J49="enviado",J49="aceptado",J49="rechazado"),L49=""),"Falta fecha de presentación",IF(AND(OR(J49="aceptado",J49="rechazado"),M49=""),"Falta fecha de respuesta",IF(AND(I49&lt;&gt;"",H49&lt;&gt;"",I49&lt;H49),"Vencimiento anterior a emisión","Lista para importar")))))</f>
         <v/>
       </c>
     </row>
@@ -1597,8 +1646,9 @@
       <c r="K50" s="51" t="n"/>
       <c r="L50" s="51" t="n"/>
       <c r="M50" s="17" t="n"/>
-      <c r="N50" s="20">
-        <f>IF(COUNTA(A50:M50)=0,"",IF(OR(A50="",B50="",C50="",E50="",I50=""),"Faltan campos obligatorios",IF(AND(I50="exportado",J50=""),"Falta fecha de exportación",IF(AND(OR(I50="enviado",I50="aceptado",I50="rechazado"),K50=""),"Falta fecha de presentación",IF(AND(OR(I50="aceptado",I50="rechazado"),L50=""),"Falta fecha de respuesta",IF(AND(H50&lt;&gt;"",G50&lt;&gt;"",H50&lt;G50),"Vencimiento anterior a emisión","Lista para importar"))))))</f>
+      <c r="N50" s="20" t="n"/>
+      <c r="O50">
+        <f>IF(COUNTA(A50:M50)=0,"",IF(OR(A50="",B50="",C50="",E50="",J50=""),"Faltan campos obligatorios",IF(AND(J50="exportado",K50=""),"Falta fecha de exportación",IF(AND(OR(J50="enviado",J50="aceptado",J50="rechazado"),L50=""),"Falta fecha de presentación",IF(AND(OR(J50="aceptado",J50="rechazado"),M50=""),"Falta fecha de respuesta",IF(AND(I50&lt;&gt;"",H50&lt;&gt;"",I50&lt;H50),"Vencimiento anterior a emisión","Lista para importar")))))</f>
         <v/>
       </c>
     </row>
@@ -1634,7 +1684,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A5"/>
+  <dimension ref="A1:A6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1680,7 +1730,13 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="46" customHeight="1"/>
+    <row r="6" ht="46" customHeight="1">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>La columna Control es solo ayuda en Excel; no se importa al sistema.</t>
+        </is>
+      </c>
+    </row>
     <row r="7" ht="46" customHeight="1"/>
     <row r="8" ht="46" customHeight="1"/>
     <row r="9" ht="46" customHeight="1"/>

</xml_diff>